<commit_message>
feat: Add Hayden case studies README and cross-case comparison (#22)
- Add comprehensive README.md for hayden_case_studies with citations
- Expand Nebraska K-12 case study to minimum depth (10 components, 16 cells, 22 deliveries)
  - Added federal oversight, state board, communities, teachers union, property assessors
  - Added circular causation: property values → assessments → TEEOSA → funding → school quality → values
  - Added ceremonial-instrumental conflict: union resistance to centralization
  - Added feedback loops: student outcomes → community demands → district accountability
- Add compare_cases.py for cross-case comparison
  - Runs analysis battery on all four case studies
  - Generates formatted comparison table with 12 metrics
  - Provides cross-case insights and summary statistics
- Add smoke tests for compare_cases.py (3 tests)
- Update repository README with case studies section
- All tests passing (708/708), mypy clean, pyflakes clean
</commit_message>
<xml_diff>
--- a/examples/hayden_case_studies/director_networks.xlsx
+++ b/examples/hayden_case_studies/director_networks.xlsx
@@ -619,7 +619,7 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>information: Mergers and acquisitions advisory services
 money: Underwriting for debt offerings</t>
@@ -761,7 +761,7 @@
           <t>Director Smith</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>authority: Board governance and strategic oversight
 information: Industry intelligence from Boeing and Business Roundtable co...</t>
@@ -770,7 +770,7 @@
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>authority: Board governance and strategic oversight
 information: Financial sector intelligence from Citigroup connections</t>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>authority: Board governance and strategic oversight
 information: Financial sector intelligence from JP Morgan connections</t>
@@ -861,37 +861,37 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Goldman Sachs</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs provides M&amp;A advisory to AT&amp;T</t>
+          <t>GE compensates Director Jones for board service</t>
         </is>
       </c>
       <c r="D2" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
+          <t>JP Morgan Chase</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
           <t>General Electric</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Director Jones</t>
-        </is>
-      </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>GE compensates Director Jones for board service</t>
+          <t>JP Morgan provides capital and investment banking to GE</t>
         </is>
       </c>
       <c r="D3" s="9" t="n">
@@ -901,17 +901,17 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>U.S. Chamber provides advocacy for General Electric</t>
+          <t>JP Morgan compensates Director Jones for board service</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
@@ -921,37 +921,37 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>U.S. Chamber provides advocacy for AT&amp;T</t>
+          <t>Director Jones serves on GE board providing governance and banking expertise</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>U.S. Chamber provides advocacy for Citigroup</t>
+          <t>Director Jones serves on JP Morgan board providing governance oversight</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
@@ -966,32 +966,32 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Director Jones serves on GE board providing governance and banking expertise</t>
+          <t>Director Jones participates in U.S. Chamber banking policy</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Director Jones participates in U.S. Chamber banking policy</t>
+          <t>Director Smith participates in Business Roundtable policy formation</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
@@ -1001,21 +1001,21 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Director Jones serves on JP Morgan board providing governance oversight</t>
+          <t>Director Smith serves on Citigroup board providing governance oversight</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1026,56 +1026,56 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Director Smith participates in Business Roundtable policy formation</t>
+          <t>Director Smith serves on Boeing board providing governance and financial expertise</t>
         </is>
       </c>
       <c r="D10" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Director Smith serves on Citigroup board providing governance oversight</t>
+          <t>Business Roundtable coordinates policy positions for General Electric</t>
         </is>
       </c>
       <c r="D11" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Director Smith serves on Boeing board providing governance and financial expertise</t>
+          <t>Business Roundtable coordinates policy positions for JP Morgan Chase</t>
         </is>
       </c>
       <c r="D12" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Business Roundtable coordinates policy positions for General Electric</t>
+          <t>Business Roundtable coordinates policy positions for Citigroup</t>
         </is>
       </c>
       <c r="D13" s="9" t="n">
@@ -1106,12 +1106,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Business Roundtable coordinates policy positions for AT&amp;T</t>
+          <t>Business Roundtable coordinates policy positions for Boeing</t>
         </is>
       </c>
       <c r="D14" s="9" t="n">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Business Roundtable coordinates policy positions for Citigroup</t>
+          <t>Business Roundtable coordinates policy positions for AT&amp;T</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -1141,37 +1141,37 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Business Roundtable coordinates policy positions for Boeing</t>
+          <t>Goldman Sachs provides M&amp;A advisory to AT&amp;T</t>
         </is>
       </c>
       <c r="D16" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Business Roundtable coordinates policy positions for JP Morgan Chase</t>
+          <t>U.S. Chamber provides advocacy for General Electric</t>
         </is>
       </c>
       <c r="D17" s="9" t="n">
@@ -1181,47 +1181,47 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
+          <t>U.S. Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
           <t>Citigroup</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Director Smith</t>
-        </is>
-      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Citigroup compensates Director Smith for board service</t>
+          <t>U.S. Chamber provides advocacy for Citigroup</t>
         </is>
       </c>
       <c r="D18" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Citigroup provides credit facility to Boeing for production financing</t>
+          <t>U.S. Chamber provides advocacy for AT&amp;T</t>
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -1231,47 +1231,47 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Boeing compensates Director Smith for board service</t>
+          <t>Citigroup compensates Director Smith for board service</t>
         </is>
       </c>
       <c r="D20" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>JP Morgan provides capital and investment banking to GE</t>
+          <t>Citigroup provides credit facility to Boeing for production financing</t>
         </is>
       </c>
       <c r="D21" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>JP Morgan compensates Director Jones for board service</t>
+          <t>Boeing compensates Director Smith for board service</t>
         </is>
       </c>
       <c r="D22" s="9" t="n">
@@ -1353,41 +1353,51 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Goldman Sachs</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Mergers and acquisitions advisory services</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="8" t="n"/>
-      <c r="G2" s="8" t="n"/>
+          <t>Annual board compensation and stock options</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="n">
+        <v>325000</v>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>USD/year</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
       <c r="H2" s="10" t="n"/>
       <c r="I2" s="10" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Goldman Sachs</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -1397,11 +1407,11 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Underwriting for debt offerings</t>
+          <t>$5B revolving credit and investment banking services</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
-        <v>3000000000</v>
+        <v>5000000000</v>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
@@ -1410,18 +1420,18 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="H3" s="10" t="n"/>
       <c r="I3" s="10" t="n">
-        <v>0.85</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1440,7 +1450,7 @@
         </is>
       </c>
       <c r="E4" s="10" t="n">
-        <v>325000</v>
+        <v>400000</v>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
@@ -1460,7 +1470,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1470,12 +1480,12 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Advocacy positions and legislative recommendations</t>
+          <t>Board governance and strategic oversight</t>
         </is>
       </c>
       <c r="E5" s="10" t="n"/>
@@ -1483,28 +1493,28 @@
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="10" t="n"/>
       <c r="I5" s="10" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>AT&amp;T</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Advocacy positions and legislative recommendations</t>
+          <t>Financial sector intelligence from JP Morgan connections</t>
         </is>
       </c>
       <c r="E6" s="10" t="n"/>
@@ -1512,28 +1522,28 @@
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="10" t="n"/>
       <c r="I6" s="10" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Director Jones</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>rule</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Advocacy positions and legislative recommendations</t>
+          <t>Board governance and strategic oversight</t>
         </is>
       </c>
       <c r="E7" s="10" t="n"/>
@@ -1541,7 +1551,7 @@
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="10" t="n"/>
       <c r="I7" s="10" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1552,17 +1562,17 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Board governance and strategic oversight</t>
+          <t>Banking sector perspective and policy input</t>
         </is>
       </c>
       <c r="E8" s="10" t="n"/>
@@ -1570,18 +1580,18 @@
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="10" t="n"/>
       <c r="I8" s="10" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -1591,7 +1601,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Financial sector intelligence from JP Morgan connections</t>
+          <t>Industry intelligence and policy input</t>
         </is>
       </c>
       <c r="E9" s="10" t="n"/>
@@ -1605,22 +1615,22 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>U.S. Chamber of Commerce</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Banking sector perspective and policy input</t>
+          <t>Board governance and strategic oversight</t>
         </is>
       </c>
       <c r="E10" s="10" t="n"/>
@@ -1628,28 +1638,28 @@
       <c r="G10" s="8" t="n"/>
       <c r="H10" s="10" t="n"/>
       <c r="I10" s="10" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Board governance and strategic oversight</t>
+          <t>Industry intelligence from Boeing and Business Roundtable connections</t>
         </is>
       </c>
       <c r="E11" s="10" t="n"/>
@@ -1657,7 +1667,7 @@
       <c r="G11" s="8" t="n"/>
       <c r="H11" s="10" t="n"/>
       <c r="I11" s="10" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="12">
@@ -1668,17 +1678,17 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>authority</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Industry intelligence and policy input</t>
+          <t>Board governance and strategic oversight</t>
         </is>
       </c>
       <c r="E12" s="10" t="n"/>
@@ -1686,7 +1696,7 @@
       <c r="G12" s="8" t="n"/>
       <c r="H12" s="10" t="n"/>
       <c r="I12" s="10" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1697,17 +1707,17 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Board governance and strategic oversight</t>
+          <t>Financial sector intelligence from Citigroup connections</t>
         </is>
       </c>
       <c r="E13" s="10" t="n"/>
@@ -1715,18 +1725,18 @@
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="10" t="n"/>
       <c r="I13" s="10" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -1736,7 +1746,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Industry intelligence from Boeing and Business Roundtable connections</t>
+          <t>Coordinated policy positions on corporate governance and regulation</t>
         </is>
       </c>
       <c r="E14" s="10" t="n"/>
@@ -1744,28 +1754,28 @@
       <c r="G14" s="8" t="n"/>
       <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>JP Morgan Chase</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Board governance and strategic oversight</t>
+          <t>Coordinated policy positions on corporate governance and regulation</t>
         </is>
       </c>
       <c r="E15" s="10" t="n"/>
@@ -1773,18 +1783,18 @@
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="10" t="n"/>
       <c r="I15" s="10" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>Business Roundtable</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -1794,7 +1804,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Financial sector intelligence from Citigroup connections</t>
+          <t>Coordinated policy positions on corporate governance and regulation</t>
         </is>
       </c>
       <c r="E16" s="10" t="n"/>
@@ -1802,7 +1812,7 @@
       <c r="G16" s="8" t="n"/>
       <c r="H16" s="10" t="n"/>
       <c r="I16" s="10" t="n">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="17">
@@ -1813,7 +1823,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -1866,12 +1876,12 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -1881,7 +1891,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Coordinated policy positions on corporate governance and regulation</t>
+          <t>Mergers and acquisitions advisory services</t>
         </is>
       </c>
       <c r="E19" s="10" t="n"/>
@@ -1889,57 +1899,67 @@
       <c r="G19" s="8" t="n"/>
       <c r="H19" s="10" t="n"/>
       <c r="I19" s="10" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>Goldman Sachs</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>money</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Coordinated policy positions on corporate governance and regulation</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="8" t="n"/>
-      <c r="G20" s="8" t="n"/>
+          <t>Underwriting for debt offerings</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>3000000000</v>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>annual</t>
+        </is>
+      </c>
       <c r="H20" s="10" t="n"/>
       <c r="I20" s="10" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Business Roundtable</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>General Electric</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Coordinated policy positions on corporate governance and regulation</t>
+          <t>Advocacy positions and legislative recommendations</t>
         </is>
       </c>
       <c r="E21" s="10" t="n"/>
@@ -1947,67 +1967,57 @@
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="10" t="n"/>
       <c r="I21" s="10" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
+          <t>U.S. Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
           <t>Citigroup</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Director Smith</t>
-        </is>
-      </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Annual board compensation and stock options</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="n">
-        <v>350000</v>
-      </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>USD/year</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>annual</t>
-        </is>
-      </c>
+          <t>Advocacy positions and legislative recommendations</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
       <c r="H22" s="10" t="n"/>
       <c r="I22" s="10" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Citigroup</t>
+          <t>U.S. Chamber of Commerce</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Director Smith</t>
+          <t>AT&amp;T</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>information</t>
+          <t>rule</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Access to confidential financial data and strategic plans</t>
+          <t>Advocacy positions and legislative recommendations</t>
         </is>
       </c>
       <c r="E23" s="10" t="n"/>
@@ -2015,7 +2025,7 @@
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="10" t="n"/>
       <c r="I23" s="10" t="n">
-        <v>0.95</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="24">
@@ -2026,7 +2036,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -2036,25 +2046,25 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>$2.5B credit facility for aircraft production</t>
+          <t>Annual board compensation and stock options</t>
         </is>
       </c>
       <c r="E24" s="10" t="n">
-        <v>2500000000</v>
+        <v>350000</v>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>USD/year</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>continuous</t>
+          <t>annual</t>
         </is>
       </c>
       <c r="H24" s="10" t="n"/>
       <c r="I24" s="10" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -2065,7 +2075,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Boeing</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -2075,7 +2085,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Market intelligence and financial advisory</t>
+          <t>Access to confidential financial data and strategic plans</t>
         </is>
       </c>
       <c r="E25" s="10" t="n"/>
@@ -2083,20 +2093,20 @@
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="10" t="n"/>
       <c r="I25" s="10" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
+          <t>Citigroup</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
           <t>Boeing</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Director Smith</t>
-        </is>
-      </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
           <t>money</t>
@@ -2104,75 +2114,65 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Annual board compensation and stock options</t>
+          <t>$2.5B credit facility for aircraft production</t>
         </is>
       </c>
       <c r="E26" s="10" t="n">
-        <v>300000</v>
+        <v>2500000000</v>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>USD/year</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>annual</t>
+          <t>continuous</t>
         </is>
       </c>
       <c r="H26" s="10" t="n"/>
       <c r="I26" s="10" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Citigroup</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>General Electric</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>money</t>
+          <t>information</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>$5B revolving credit and investment banking services</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>5000000000</v>
-      </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>continuous</t>
-        </is>
-      </c>
+          <t>Market intelligence and financial advisory</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
       <c r="H27" s="10" t="n"/>
       <c r="I27" s="10" t="n">
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>JP Morgan Chase</t>
+          <t>Boeing</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Director Jones</t>
+          <t>Director Smith</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="E28" s="10" t="n">
-        <v>400000</v>
+        <v>300000</v>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>

</xml_diff>